<commit_message>
fix(7.2): the examples after their reviews, and D302, D303
Drift (D302, D303): formula_workbook.py and export_clean.py named only the empty
workbook as the file main ships but can't rebuild, copied byte for byte; the
examples are too. The code review: example 2's map called ROLLUP's row a
Subtotal row, as the glossary says; the Power Query and Hive sheets share one
writer; copilot_files.py no longer drops the empty workbook's result. The
beginner reader: Excel's Load To can't fill an existing Table, so example 3's
steps delete the typed-in Table, load the query in its place and type the
hours column again; its map says why Table ok_runs is a final; the Hive sheet
names all five files and says to delete the Power Query sheet too; the README
says example 3's queries are added by hand.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copilot/examples/01_formulas.xlsx
+++ b/copilot/examples/01_formulas.xlsx
@@ -1154,10 +1154,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What Copilot gives with files 11 and 12 loaded: the map, then a query per final. Fill in &lt;database&gt; with your database's name. Delete this sheet before you try the workbook on Copilot yourself.</t>
-        </is>
-      </c>
-    </row>
+          <t>What Copilot gives with files 11, 12, 03, 04 and 05 loaded: the map, then a query per final. Fill in &lt;database&gt; with your database's name. Delete this sheet, and the Power Query sheet if there is one, before you try the workbook on Copilot yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1165,6 +1166,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>

</xml_diff>